<commit_message>
docs: tb_report_job 을 스키마 문서 4종에 반영해 schema-docs 게이트를 되살린다 (#722)
PR #703 이 tb_report_job 을 만들면서 스키마 문서를 갱신하지 않아
required 게이트 schema-docs(central 전용)가 빨간불이었다. 개인 워크트리
pre-push 에는 없는 게이트라 로컬은 전부 통과한 것처럼 보였다.

- 데이터베이스.md: 요약표에 행 추가 + §7 인프라에 컬럼별 설명 절 신설
  (근거는 20260820143044_report_job.sql 의 DDL 과 server/src/report_job.php)
- erd.puml: "피드 운영 · 인증 · 감사" package 에 엔티티 추가,
  tb_host·tb_user 와 실선(실제 FK) 관계선 연결
- erd.svg · 테이블명세서.xlsx: 생성기로 재생성

PR #719 의 레이아웃 결정(linetype ortho 없음, -[hidden]- 보조선)은 그대로 뒀다.
폭은 2547 -> 2558 로 목표(<=2700) 안이다. 보조선을 하나 더 붙여 세로를 줄이는
3안을 실측했으나 폭이 2928~3180 으로 튀어 채택하지 않았다.
</commit_message>
<xml_diff>
--- a/docs/specs/테이블명세서.xlsx
+++ b/docs/specs/테이블명세서.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1686,12 +1686,12 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>tb_schema_migrations</t>
+          <t>tb_report_job</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>적용된 마이그레이션 기록</t>
+          <t>AI 보고서 작업(외부 작업큐)의 우리 쪽 대장 — 요청자·상태·결과</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -1701,41 +1701,41 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>△ created_at/updated_at</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>tb_discovery_target</t>
+          <t>tb_schema_migrations</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>관리자가 등록한 스캔 대역(자연키 `cidr`)</t>
+          <t>적용된 마이그레이션 기록</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>§8 자산 탐색</t>
+          <t>§7 인프라</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>tb_discovery_run</t>
+          <t>tb_discovery_target</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>대역 스윕 1회분 실행 이력과 집계</t>
+          <t>관리자가 등록한 스캔 대역(자연키 `cidr`)</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -1752,12 +1752,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>tb_discovered_asset</t>
+          <t>tb_discovery_run</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>발견한 IP(대역 기준 누적) — `host_id` NULL = 섀도우 IT 후보</t>
+          <t>대역 스윕 1회분 실행 이력과 집계</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -1774,20 +1774,42 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
+          <t>tb_discovered_asset</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>발견한 IP(대역 기준 누적) — `host_id` NULL = 섀도우 IT 후보</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>§8 자산 탐색</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
           <t>tb_discovered_port</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>발견 IP 의 열린 포트(open 만 저장)</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C62" s="3" t="inlineStr">
         <is>
           <t>§8 자산 탐색</t>
         </is>
       </c>
-      <c r="D61" s="3" t="inlineStr">
+      <c r="D62" s="3" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -1804,7 +1826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G699"/>
+  <dimension ref="A1:G710"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -21709,17 +21731,17 @@
     <row r="647">
       <c r="A647" s="4" t="inlineStr">
         <is>
-          <t>tb_schema_migrations</t>
+          <t>tb_report_job</t>
         </is>
       </c>
       <c r="B647" s="4" t="inlineStr">
         <is>
-          <t>filename</t>
+          <t>report_job_id</t>
         </is>
       </c>
       <c r="C647" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(191)</t>
+          <t>BIGINT UNSIGNED</t>
         </is>
       </c>
       <c r="D647" s="5" t="inlineStr">
@@ -21732,23 +21754,27 @@
           <t>PK</t>
         </is>
       </c>
-      <c r="F647" s="5" t="inlineStr"/>
+      <c r="F647" s="5" t="inlineStr">
+        <is>
+          <t>AUTO_INCREMENT</t>
+        </is>
+      </c>
       <c r="G647" s="3" t="inlineStr"/>
     </row>
     <row r="648">
       <c r="A648" s="4" t="inlineStr">
         <is>
-          <t>tb_schema_migrations</t>
+          <t>tb_report_job</t>
         </is>
       </c>
       <c r="B648" s="4" t="inlineStr">
         <is>
-          <t>applied_at</t>
+          <t>host_id</t>
         </is>
       </c>
       <c r="C648" s="5" t="inlineStr">
         <is>
-          <t>DATETIME</t>
+          <t>BIGINT UNSIGNED</t>
         </is>
       </c>
       <c r="D648" s="5" t="inlineStr">
@@ -21758,25 +21784,25 @@
       </c>
       <c r="E648" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F648" s="5" t="inlineStr">
-        <is>
-          <t>CURRENT_TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="G648" s="3" t="inlineStr"/>
+          <t>MUL</t>
+        </is>
+      </c>
+      <c r="F648" s="5" t="inlineStr"/>
+      <c r="G648" s="3" t="inlineStr">
+        <is>
+          <t>보고서를 만든 대상 호스트(tb_host.host_id). 호스트를 하드 삭제하면 ON DELETE CASCADE 로 그 호스트의 job 이력도 함께 사라진다. 인덱스 (host_id, report_job_id) 가 호스트 상세의 "보고서 이력(최신순)" 조회와 정렬을 함께 덮는다(AUTO_INCREMENT PK 라 역순이 곧 최신순).</t>
+        </is>
+      </c>
     </row>
     <row r="649">
       <c r="A649" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_target</t>
+          <t>tb_report_job</t>
         </is>
       </c>
       <c r="B649" s="4" t="inlineStr">
         <is>
-          <t>discovery_target_id</t>
+          <t>external_job_id</t>
         </is>
       </c>
       <c r="C649" s="5" t="inlineStr">
@@ -21791,30 +21817,30 @@
       </c>
       <c r="E649" s="5" t="inlineStr">
         <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F649" s="5" t="inlineStr">
-        <is>
-          <t>AUTO_INCREMENT</t>
-        </is>
-      </c>
-      <c r="G649" s="3" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F649" s="5" t="inlineStr"/>
+      <c r="G649" s="3" t="inlineStr">
+        <is>
+          <t>외부 API 가 발급한 job 번호(POST /jobs/ 응답의 id). 우리 PK 와는 다른 값이라 따로 담는다 — 상태 조회(GET /jobs/{external_job_id})가 이 값으로 나간다.</t>
+        </is>
+      </c>
     </row>
     <row r="650">
       <c r="A650" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_target</t>
+          <t>tb_report_job</t>
         </is>
       </c>
       <c r="B650" s="4" t="inlineStr">
         <is>
-          <t>cidr</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C650" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(64)</t>
+          <t>VARCHAR(32)</t>
         </is>
       </c>
       <c r="D650" s="5" t="inlineStr">
@@ -21824,30 +21850,34 @@
       </c>
       <c r="E650" s="5" t="inlineStr">
         <is>
-          <t>UNI</t>
-        </is>
-      </c>
-      <c r="F650" s="5" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F650" s="5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
       <c r="G650" s="3" t="inlineStr">
         <is>
-          <t>예: 10.3.142.0/24</t>
+          <t>외부 API 가 준 상태 문자열 원문(32자로 자름, 기본값 PENDING). 외부에서 확정받은 어휘는 PENDING·PROCESSING·SUCCESS·FAILED 네 가지지만 우리가 어휘를 정의하지는 않는다 — server/src/report_job.php 의 VG_REPORT_STATUS_DONE(완료로 볼 값)·VG_REPORT_STATUS_FAILED(실패로 볼 값) 두 목록만 두고 어느 쪽에도 없는 값은 진행 중으로 읽는다(모르는 값을 완료로 읽으면 안 끝난 job 의 빈 결과를 보여주게 된다).</t>
         </is>
       </c>
     </row>
     <row r="651">
       <c r="A651" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_target</t>
+          <t>tb_report_job</t>
         </is>
       </c>
       <c r="B651" s="4" t="inlineStr">
         <is>
-          <t>ports</t>
+          <t>result</t>
         </is>
       </c>
       <c r="C651" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(1024)</t>
+          <t>MEDIUMTEXT</t>
         </is>
       </c>
       <c r="D651" s="5" t="inlineStr">
@@ -21863,24 +21893,24 @@
       <c r="F651" s="5" t="inlineStr"/>
       <c r="G651" s="3" t="inlineStr">
         <is>
-          <t>2단계에서 두드릴 포트 목록(콤마·범위). NULL 이면 기본 세트를 쓴다 — 대역마다 다른 포트를 보고 싶을 때만 채운다.</t>
+          <t>외부가 준 결과 본문(MEDIUMTEXT). 형식이 정해지지 않아 화면은 plain text 로만 그린다(vg_h() 이스케이프). 결과가 파일 링크면 그 외부 주소를 화면에 내리지 않고 우리 프록시(report-download.php?job=&lt;report_job_id&gt;)가 대신 받아 내려준다(SSRF 방지 — 목적지는 서버가 이 컬럼에서 만든다). NULL = 아직 결과 없음.</t>
         </is>
       </c>
     </row>
     <row r="652">
       <c r="A652" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_target</t>
+          <t>tb_report_job</t>
         </is>
       </c>
       <c r="B652" s="4" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>error_message</t>
         </is>
       </c>
       <c r="C652" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(255)</t>
+          <t>VARCHAR(1000)</t>
         </is>
       </c>
       <c r="D652" s="5" t="inlineStr">
@@ -21894,55 +21924,59 @@
         </is>
       </c>
       <c r="F652" s="5" t="inlineStr"/>
-      <c r="G652" s="3" t="inlineStr"/>
+      <c r="G652" s="3" t="inlineStr">
+        <is>
+          <t>외부 API 가 준 error_message(1000자로 자름). 우리 내부 예외 원문은 넣지 않는다 — 스택트레이스·SQL·경로를 사용자 화면에 노출하지 않는 원칙 그대로다. NULL = 오류 없음.</t>
+        </is>
+      </c>
     </row>
     <row r="653">
       <c r="A653" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_target</t>
+          <t>tb_report_job</t>
         </is>
       </c>
       <c r="B653" s="4" t="inlineStr">
         <is>
-          <t>enabled</t>
+          <t>requested_user_id</t>
         </is>
       </c>
       <c r="C653" s="5" t="inlineStr">
         <is>
-          <t>TINYINT(1)</t>
+          <t>BIGINT UNSIGNED</t>
         </is>
       </c>
       <c r="D653" s="5" t="inlineStr">
         <is>
-          <t>아니오</t>
+          <t>예</t>
         </is>
       </c>
       <c r="E653" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F653" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G653" s="3" t="inlineStr"/>
+          <t>MUL</t>
+        </is>
+      </c>
+      <c r="F653" s="5" t="inlineStr"/>
+      <c r="G653" s="3" t="inlineStr">
+        <is>
+          <t>생성 버튼을 누른 사용자(tb_user.user_id). 계정이 지워져도 이력은 남겨야 하므로 ON DELETE SET NULL 이고, 그래서 NULL = 요청자 계정이 이미 삭제된 행이다. 이력 목록은 이 값을 tb_user 와 LEFT JOIN 해 사용자명을 보여준다.</t>
+        </is>
+      </c>
     </row>
     <row r="654">
       <c r="A654" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_target</t>
+          <t>tb_report_job</t>
         </is>
       </c>
       <c r="B654" s="4" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>external_created_at</t>
         </is>
       </c>
       <c r="C654" s="5" t="inlineStr">
         <is>
-          <t>BIGINT UNSIGNED</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D654" s="5" t="inlineStr">
@@ -21958,19 +21992,19 @@
       <c r="F654" s="5" t="inlineStr"/>
       <c r="G654" s="3" t="inlineStr">
         <is>
-          <t>tb_user.user_id (FK 없음)</t>
+          <t>외부가 준 job 생성·완료 시각을 Y-m-d H:i:s 로 옮긴 값이다 — 우리 created_at 과 다른 저쪽 시계이고, 외부가 안 줬거나 아직 안 끝났으면 NULL 이다.</t>
         </is>
       </c>
     </row>
     <row r="655">
       <c r="A655" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_target</t>
+          <t>tb_report_job</t>
         </is>
       </c>
       <c r="B655" s="4" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>external_finished_at</t>
         </is>
       </c>
       <c r="C655" s="5" t="inlineStr">
@@ -21980,7 +22014,7 @@
       </c>
       <c r="D655" s="5" t="inlineStr">
         <is>
-          <t>아니오</t>
+          <t>예</t>
         </is>
       </c>
       <c r="E655" s="5" t="inlineStr">
@@ -21988,22 +22022,22 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F655" s="5" t="inlineStr">
-        <is>
-          <t>CURRENT_TIMESTAMP</t>
-        </is>
-      </c>
-      <c r="G655" s="3" t="inlineStr"/>
+      <c r="F655" s="5" t="inlineStr"/>
+      <c r="G655" s="3" t="inlineStr">
+        <is>
+          <t>외부가 준 job 생성·완료 시각을 Y-m-d H:i:s 로 옮긴 값이다 — 우리 created_at 과 다른 저쪽 시계이고, 외부가 안 줬거나 아직 안 끝났으면 NULL 이다.</t>
+        </is>
+      </c>
     </row>
     <row r="656">
       <c r="A656" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_target</t>
+          <t>tb_report_job</t>
         </is>
       </c>
       <c r="B656" s="4" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C656" s="5" t="inlineStr">
@@ -22023,25 +22057,29 @@
       </c>
       <c r="F656" s="5" t="inlineStr">
         <is>
-          <t>CURRENT_TIMESTAMP (ON UPDATE)</t>
-        </is>
-      </c>
-      <c r="G656" s="3" t="inlineStr"/>
+          <t>CURRENT_TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="G656" s="3" t="inlineStr">
+        <is>
+          <t>우리 표에 남긴 시각(요청 시점 / 마지막 폴링 반영 시점). is_deleted·deleted_at 은 두지 않는다 — 사람이 지우는 화면이 없어 삭제 경로 자체가 없다(tb_finding_status 와 같은 판단).</t>
+        </is>
+      </c>
     </row>
     <row r="657">
       <c r="A657" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_target</t>
+          <t>tb_report_job</t>
         </is>
       </c>
       <c r="B657" s="4" t="inlineStr">
         <is>
-          <t>is_deleted</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C657" s="5" t="inlineStr">
         <is>
-          <t>TINYINT(1)</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D657" s="5" t="inlineStr">
@@ -22056,35 +22094,39 @@
       </c>
       <c r="F657" s="5" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G657" s="3" t="inlineStr"/>
+          <t>CURRENT_TIMESTAMP (ON UPDATE)</t>
+        </is>
+      </c>
+      <c r="G657" s="3" t="inlineStr">
+        <is>
+          <t>우리 표에 남긴 시각(요청 시점 / 마지막 폴링 반영 시점). is_deleted·deleted_at 은 두지 않는다 — 사람이 지우는 화면이 없어 삭제 경로 자체가 없다(tb_finding_status 와 같은 판단).</t>
+        </is>
+      </c>
     </row>
     <row r="658">
       <c r="A658" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_target</t>
+          <t>tb_schema_migrations</t>
         </is>
       </c>
       <c r="B658" s="4" t="inlineStr">
         <is>
-          <t>deleted_at</t>
+          <t>filename</t>
         </is>
       </c>
       <c r="C658" s="5" t="inlineStr">
         <is>
-          <t>DATETIME</t>
+          <t>VARCHAR(191)</t>
         </is>
       </c>
       <c r="D658" s="5" t="inlineStr">
         <is>
-          <t>예</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="E658" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="F658" s="5" t="inlineStr"/>
@@ -22093,17 +22135,17 @@
     <row r="659">
       <c r="A659" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_run</t>
+          <t>tb_schema_migrations</t>
         </is>
       </c>
       <c r="B659" s="4" t="inlineStr">
         <is>
-          <t>discovery_run_id</t>
+          <t>applied_at</t>
         </is>
       </c>
       <c r="C659" s="5" t="inlineStr">
         <is>
-          <t>BIGINT UNSIGNED</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D659" s="5" t="inlineStr">
@@ -22113,12 +22155,12 @@
       </c>
       <c r="E659" s="5" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F659" s="5" t="inlineStr">
         <is>
-          <t>AUTO_INCREMENT</t>
+          <t>CURRENT_TIMESTAMP</t>
         </is>
       </c>
       <c r="G659" s="3" t="inlineStr"/>
@@ -22126,7 +22168,7 @@
     <row r="660">
       <c r="A660" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_run</t>
+          <t>tb_discovery_target</t>
         </is>
       </c>
       <c r="B660" s="4" t="inlineStr">
@@ -22146,26 +22188,30 @@
       </c>
       <c r="E660" s="5" t="inlineStr">
         <is>
-          <t>MUL</t>
-        </is>
-      </c>
-      <c r="F660" s="5" t="inlineStr"/>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F660" s="5" t="inlineStr">
+        <is>
+          <t>AUTO_INCREMENT</t>
+        </is>
+      </c>
       <c r="G660" s="3" t="inlineStr"/>
     </row>
     <row r="661">
       <c r="A661" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_run</t>
+          <t>tb_discovery_target</t>
         </is>
       </c>
       <c r="B661" s="4" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>cidr</t>
         </is>
       </c>
       <c r="C661" s="5" t="inlineStr">
         <is>
-          <t>ENUM('PENDING','RUNNING','DONE','FAILED')</t>
+          <t>VARCHAR(64)</t>
         </is>
       </c>
       <c r="D661" s="5" t="inlineStr">
@@ -22175,30 +22221,30 @@
       </c>
       <c r="E661" s="5" t="inlineStr">
         <is>
-          <t>MUL</t>
-        </is>
-      </c>
-      <c r="F661" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="G661" s="3" t="inlineStr"/>
+          <t>UNI</t>
+        </is>
+      </c>
+      <c r="F661" s="5" t="inlineStr"/>
+      <c r="G661" s="3" t="inlineStr">
+        <is>
+          <t>예: 10.3.142.0/24</t>
+        </is>
+      </c>
     </row>
     <row r="662">
       <c r="A662" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_run</t>
+          <t>tb_discovery_target</t>
         </is>
       </c>
       <c r="B662" s="4" t="inlineStr">
         <is>
-          <t>started_at</t>
+          <t>ports</t>
         </is>
       </c>
       <c r="C662" s="5" t="inlineStr">
         <is>
-          <t>DATETIME</t>
+          <t>VARCHAR(1024)</t>
         </is>
       </c>
       <c r="D662" s="5" t="inlineStr">
@@ -22212,22 +22258,26 @@
         </is>
       </c>
       <c r="F662" s="5" t="inlineStr"/>
-      <c r="G662" s="3" t="inlineStr"/>
+      <c r="G662" s="3" t="inlineStr">
+        <is>
+          <t>2단계에서 두드릴 포트 목록(콤마·범위). NULL 이면 기본 세트를 쓴다 — 대역마다 다른 포트를 보고 싶을 때만 채운다.</t>
+        </is>
+      </c>
     </row>
     <row r="663">
       <c r="A663" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_run</t>
+          <t>tb_discovery_target</t>
         </is>
       </c>
       <c r="B663" s="4" t="inlineStr">
         <is>
-          <t>finished_at</t>
+          <t>label</t>
         </is>
       </c>
       <c r="C663" s="5" t="inlineStr">
         <is>
-          <t>DATETIME</t>
+          <t>VARCHAR(255)</t>
         </is>
       </c>
       <c r="D663" s="5" t="inlineStr">
@@ -22246,17 +22296,17 @@
     <row r="664">
       <c r="A664" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_run</t>
+          <t>tb_discovery_target</t>
         </is>
       </c>
       <c r="B664" s="4" t="inlineStr">
         <is>
-          <t>ip_total</t>
+          <t>enabled</t>
         </is>
       </c>
       <c r="C664" s="5" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>TINYINT(1)</t>
         </is>
       </c>
       <c r="D664" s="5" t="inlineStr">
@@ -22271,34 +22321,30 @@
       </c>
       <c r="F664" s="5" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G664" s="3" t="inlineStr">
-        <is>
-          <t>대역의 IP 수</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G664" s="3" t="inlineStr"/>
     </row>
     <row r="665">
       <c r="A665" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_run</t>
+          <t>tb_discovery_target</t>
         </is>
       </c>
       <c r="B665" s="4" t="inlineStr">
         <is>
-          <t>ip_alive</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="C665" s="5" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>BIGINT UNSIGNED</t>
         </is>
       </c>
       <c r="D665" s="5" t="inlineStr">
         <is>
-          <t>아니오</t>
+          <t>예</t>
         </is>
       </c>
       <c r="E665" s="5" t="inlineStr">
@@ -22306,31 +22352,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F665" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="F665" s="5" t="inlineStr"/>
       <c r="G665" s="3" t="inlineStr">
         <is>
-          <t>1단계에서 살아있다고 판정된 수</t>
+          <t>tb_user.user_id (FK 없음)</t>
         </is>
       </c>
     </row>
     <row r="666">
       <c r="A666" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_run</t>
+          <t>tb_discovery_target</t>
         </is>
       </c>
       <c r="B666" s="4" t="inlineStr">
         <is>
-          <t>port_checked</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C666" s="5" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D666" s="5" t="inlineStr">
@@ -22345,29 +22387,25 @@
       </c>
       <c r="F666" s="5" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G666" s="3" t="inlineStr">
-        <is>
-          <t>실제 시도한 (IP,포트) 조합 수 — 성능 근거</t>
-        </is>
-      </c>
+          <t>CURRENT_TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="G666" s="3" t="inlineStr"/>
     </row>
     <row r="667">
       <c r="A667" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_run</t>
+          <t>tb_discovery_target</t>
         </is>
       </c>
       <c r="B667" s="4" t="inlineStr">
         <is>
-          <t>open_total</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C667" s="5" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D667" s="5" t="inlineStr">
@@ -22382,7 +22420,7 @@
       </c>
       <c r="F667" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>CURRENT_TIMESTAMP (ON UPDATE)</t>
         </is>
       </c>
       <c r="G667" s="3" t="inlineStr"/>
@@ -22390,22 +22428,22 @@
     <row r="668">
       <c r="A668" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_run</t>
+          <t>tb_discovery_target</t>
         </is>
       </c>
       <c r="B668" s="4" t="inlineStr">
         <is>
-          <t>elapsed_seconds</t>
+          <t>is_deleted</t>
         </is>
       </c>
       <c r="C668" s="5" t="inlineStr">
         <is>
-          <t>DECIMAL(8,2)</t>
+          <t>TINYINT(1)</t>
         </is>
       </c>
       <c r="D668" s="5" t="inlineStr">
         <is>
-          <t>예</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="E668" s="5" t="inlineStr">
@@ -22413,23 +22451,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F668" s="5" t="inlineStr"/>
+      <c r="F668" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="G668" s="3" t="inlineStr"/>
     </row>
     <row r="669">
       <c r="A669" s="4" t="inlineStr">
         <is>
-          <t>tb_discovery_run</t>
+          <t>tb_discovery_target</t>
         </is>
       </c>
       <c r="B669" s="4" t="inlineStr">
         <is>
-          <t>error_text</t>
+          <t>deleted_at</t>
         </is>
       </c>
       <c r="C669" s="5" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D669" s="5" t="inlineStr">
@@ -22453,7 +22495,7 @@
       </c>
       <c r="B670" s="4" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>discovery_run_id</t>
         </is>
       </c>
       <c r="C670" s="5" t="inlineStr">
@@ -22463,20 +22505,20 @@
       </c>
       <c r="D670" s="5" t="inlineStr">
         <is>
-          <t>예</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="E670" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F670" s="5" t="inlineStr"/>
-      <c r="G670" s="3" t="inlineStr">
-        <is>
-          <t>tb_user.user_id (FK 없음)</t>
-        </is>
-      </c>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F670" s="5" t="inlineStr">
+        <is>
+          <t>AUTO_INCREMENT</t>
+        </is>
+      </c>
+      <c r="G670" s="3" t="inlineStr"/>
     </row>
     <row r="671">
       <c r="A671" s="4" t="inlineStr">
@@ -22486,12 +22528,12 @@
       </c>
       <c r="B671" s="4" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>discovery_target_id</t>
         </is>
       </c>
       <c r="C671" s="5" t="inlineStr">
         <is>
-          <t>DATETIME</t>
+          <t>BIGINT UNSIGNED</t>
         </is>
       </c>
       <c r="D671" s="5" t="inlineStr">
@@ -22501,14 +22543,10 @@
       </c>
       <c r="E671" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F671" s="5" t="inlineStr">
-        <is>
-          <t>CURRENT_TIMESTAMP</t>
-        </is>
-      </c>
+          <t>MUL</t>
+        </is>
+      </c>
+      <c r="F671" s="5" t="inlineStr"/>
       <c r="G671" s="3" t="inlineStr"/>
     </row>
     <row r="672">
@@ -22519,12 +22557,12 @@
       </c>
       <c r="B672" s="4" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C672" s="5" t="inlineStr">
         <is>
-          <t>DATETIME</t>
+          <t>ENUM('PENDING','RUNNING','DONE','FAILED')</t>
         </is>
       </c>
       <c r="D672" s="5" t="inlineStr">
@@ -22534,12 +22572,12 @@
       </c>
       <c r="E672" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>MUL</t>
         </is>
       </c>
       <c r="F672" s="5" t="inlineStr">
         <is>
-          <t>CURRENT_TIMESTAMP (ON UPDATE)</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="G672" s="3" t="inlineStr"/>
@@ -22552,17 +22590,17 @@
       </c>
       <c r="B673" s="4" t="inlineStr">
         <is>
-          <t>is_deleted</t>
+          <t>started_at</t>
         </is>
       </c>
       <c r="C673" s="5" t="inlineStr">
         <is>
-          <t>TINYINT(1)</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D673" s="5" t="inlineStr">
         <is>
-          <t>아니오</t>
+          <t>예</t>
         </is>
       </c>
       <c r="E673" s="5" t="inlineStr">
@@ -22570,11 +22608,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F673" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="F673" s="5" t="inlineStr"/>
       <c r="G673" s="3" t="inlineStr"/>
     </row>
     <row r="674">
@@ -22585,7 +22619,7 @@
       </c>
       <c r="B674" s="4" t="inlineStr">
         <is>
-          <t>deleted_at</t>
+          <t>finished_at</t>
         </is>
       </c>
       <c r="C674" s="5" t="inlineStr">
@@ -22609,17 +22643,17 @@
     <row r="675">
       <c r="A675" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_asset</t>
+          <t>tb_discovery_run</t>
         </is>
       </c>
       <c r="B675" s="4" t="inlineStr">
         <is>
-          <t>discovered_asset_id</t>
+          <t>ip_total</t>
         </is>
       </c>
       <c r="C675" s="5" t="inlineStr">
         <is>
-          <t>BIGINT UNSIGNED</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D675" s="5" t="inlineStr">
@@ -22629,30 +22663,34 @@
       </c>
       <c r="E675" s="5" t="inlineStr">
         <is>
-          <t>PK</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F675" s="5" t="inlineStr">
         <is>
-          <t>AUTO_INCREMENT</t>
-        </is>
-      </c>
-      <c r="G675" s="3" t="inlineStr"/>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G675" s="3" t="inlineStr">
+        <is>
+          <t>대역의 IP 수</t>
+        </is>
+      </c>
     </row>
     <row r="676">
       <c r="A676" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_asset</t>
+          <t>tb_discovery_run</t>
         </is>
       </c>
       <c r="B676" s="4" t="inlineStr">
         <is>
-          <t>discovery_target_id</t>
+          <t>ip_alive</t>
         </is>
       </c>
       <c r="C676" s="5" t="inlineStr">
         <is>
-          <t>BIGINT UNSIGNED</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D676" s="5" t="inlineStr">
@@ -22662,26 +22700,34 @@
       </c>
       <c r="E676" s="5" t="inlineStr">
         <is>
-          <t>MUL</t>
-        </is>
-      </c>
-      <c r="F676" s="5" t="inlineStr"/>
-      <c r="G676" s="3" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F676" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G676" s="3" t="inlineStr">
+        <is>
+          <t>1단계에서 살아있다고 판정된 수</t>
+        </is>
+      </c>
     </row>
     <row r="677">
       <c r="A677" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_asset</t>
+          <t>tb_discovery_run</t>
         </is>
       </c>
       <c r="B677" s="4" t="inlineStr">
         <is>
-          <t>ip</t>
+          <t>port_checked</t>
         </is>
       </c>
       <c r="C677" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(45)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D677" s="5" t="inlineStr">
@@ -22694,28 +22740,36 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F677" s="5" t="inlineStr"/>
-      <c r="G677" s="3" t="inlineStr"/>
+      <c r="F677" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G677" s="3" t="inlineStr">
+        <is>
+          <t>실제 시도한 (IP,포트) 조합 수 — 성능 근거</t>
+        </is>
+      </c>
     </row>
     <row r="678">
       <c r="A678" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_asset</t>
+          <t>tb_discovery_run</t>
         </is>
       </c>
       <c r="B678" s="4" t="inlineStr">
         <is>
-          <t>hostname</t>
+          <t>open_total</t>
         </is>
       </c>
       <c r="C678" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(255)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D678" s="5" t="inlineStr">
         <is>
-          <t>예</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="E678" s="5" t="inlineStr">
@@ -22723,32 +22777,32 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F678" s="5" t="inlineStr"/>
-      <c r="G678" s="3" t="inlineStr">
-        <is>
-          <t>역DNS(PTR) 호스트명. NULL=조회 실패/미조회</t>
-        </is>
-      </c>
+      <c r="F678" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G678" s="3" t="inlineStr"/>
     </row>
     <row r="679">
       <c r="A679" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_asset</t>
+          <t>tb_discovery_run</t>
         </is>
       </c>
       <c r="B679" s="4" t="inlineStr">
         <is>
-          <t>first_seen</t>
+          <t>elapsed_seconds</t>
         </is>
       </c>
       <c r="C679" s="5" t="inlineStr">
         <is>
-          <t>DATETIME</t>
+          <t>DECIMAL(8,2)</t>
         </is>
       </c>
       <c r="D679" s="5" t="inlineStr">
         <is>
-          <t>아니오</t>
+          <t>예</t>
         </is>
       </c>
       <c r="E679" s="5" t="inlineStr">
@@ -22762,22 +22816,22 @@
     <row r="680">
       <c r="A680" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_asset</t>
+          <t>tb_discovery_run</t>
         </is>
       </c>
       <c r="B680" s="4" t="inlineStr">
         <is>
-          <t>last_seen</t>
+          <t>error_text</t>
         </is>
       </c>
       <c r="C680" s="5" t="inlineStr">
         <is>
-          <t>DATETIME</t>
+          <t>TEXT</t>
         </is>
       </c>
       <c r="D680" s="5" t="inlineStr">
         <is>
-          <t>아니오</t>
+          <t>예</t>
         </is>
       </c>
       <c r="E680" s="5" t="inlineStr">
@@ -22791,12 +22845,12 @@
     <row r="681">
       <c r="A681" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_asset</t>
+          <t>tb_discovery_run</t>
         </is>
       </c>
       <c r="B681" s="4" t="inlineStr">
         <is>
-          <t>last_run_id</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="C681" s="5" t="inlineStr">
@@ -22815,55 +22869,59 @@
         </is>
       </c>
       <c r="F681" s="5" t="inlineStr"/>
-      <c r="G681" s="3" t="inlineStr"/>
+      <c r="G681" s="3" t="inlineStr">
+        <is>
+          <t>tb_user.user_id (FK 없음)</t>
+        </is>
+      </c>
     </row>
     <row r="682">
       <c r="A682" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_asset</t>
+          <t>tb_discovery_run</t>
         </is>
       </c>
       <c r="B682" s="4" t="inlineStr">
         <is>
-          <t>host_id</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C682" s="5" t="inlineStr">
         <is>
-          <t>BIGINT UNSIGNED</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D682" s="5" t="inlineStr">
         <is>
-          <t>예</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="E682" s="5" t="inlineStr">
         <is>
-          <t>MUL</t>
-        </is>
-      </c>
-      <c r="F682" s="5" t="inlineStr"/>
-      <c r="G682" s="3" t="inlineStr">
-        <is>
-          <t>매칭된 기존 자산(없으면 NULL=섀도우 IT 후보)</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F682" s="5" t="inlineStr">
+        <is>
+          <t>CURRENT_TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="G682" s="3" t="inlineStr"/>
     </row>
     <row r="683">
       <c r="A683" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_asset</t>
+          <t>tb_discovery_run</t>
         </is>
       </c>
       <c r="B683" s="4" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C683" s="5" t="inlineStr">
         <is>
-          <t>ENUM('NEW','KNOWN','IGNORED')</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D683" s="5" t="inlineStr">
@@ -22878,7 +22936,7 @@
       </c>
       <c r="F683" s="5" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>CURRENT_TIMESTAMP (ON UPDATE)</t>
         </is>
       </c>
       <c r="G683" s="3" t="inlineStr"/>
@@ -22886,22 +22944,22 @@
     <row r="684">
       <c r="A684" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_asset</t>
+          <t>tb_discovery_run</t>
         </is>
       </c>
       <c r="B684" s="4" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>is_deleted</t>
         </is>
       </c>
       <c r="C684" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(500)</t>
+          <t>TINYINT(1)</t>
         </is>
       </c>
       <c r="D684" s="5" t="inlineStr">
         <is>
-          <t>예</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="E684" s="5" t="inlineStr">
@@ -22909,18 +22967,22 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F684" s="5" t="inlineStr"/>
+      <c r="F684" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="G684" s="3" t="inlineStr"/>
     </row>
     <row r="685">
       <c r="A685" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_asset</t>
+          <t>tb_discovery_run</t>
         </is>
       </c>
       <c r="B685" s="4" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>deleted_at</t>
         </is>
       </c>
       <c r="C685" s="5" t="inlineStr">
@@ -22930,7 +22992,7 @@
       </c>
       <c r="D685" s="5" t="inlineStr">
         <is>
-          <t>아니오</t>
+          <t>예</t>
         </is>
       </c>
       <c r="E685" s="5" t="inlineStr">
@@ -22938,11 +23000,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F685" s="5" t="inlineStr">
-        <is>
-          <t>CURRENT_TIMESTAMP</t>
-        </is>
-      </c>
+      <c r="F685" s="5" t="inlineStr"/>
       <c r="G685" s="3" t="inlineStr"/>
     </row>
     <row r="686">
@@ -22953,12 +23011,12 @@
       </c>
       <c r="B686" s="4" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>discovered_asset_id</t>
         </is>
       </c>
       <c r="C686" s="5" t="inlineStr">
         <is>
-          <t>DATETIME</t>
+          <t>BIGINT UNSIGNED</t>
         </is>
       </c>
       <c r="D686" s="5" t="inlineStr">
@@ -22968,12 +23026,12 @@
       </c>
       <c r="E686" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>PK</t>
         </is>
       </c>
       <c r="F686" s="5" t="inlineStr">
         <is>
-          <t>CURRENT_TIMESTAMP (ON UPDATE)</t>
+          <t>AUTO_INCREMENT</t>
         </is>
       </c>
       <c r="G686" s="3" t="inlineStr"/>
@@ -22986,12 +23044,12 @@
       </c>
       <c r="B687" s="4" t="inlineStr">
         <is>
-          <t>is_deleted</t>
+          <t>discovery_target_id</t>
         </is>
       </c>
       <c r="C687" s="5" t="inlineStr">
         <is>
-          <t>TINYINT(1)</t>
+          <t>BIGINT UNSIGNED</t>
         </is>
       </c>
       <c r="D687" s="5" t="inlineStr">
@@ -23001,14 +23059,10 @@
       </c>
       <c r="E687" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F687" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>MUL</t>
+        </is>
+      </c>
+      <c r="F687" s="5" t="inlineStr"/>
       <c r="G687" s="3" t="inlineStr"/>
     </row>
     <row r="688">
@@ -23019,17 +23073,17 @@
       </c>
       <c r="B688" s="4" t="inlineStr">
         <is>
-          <t>deleted_at</t>
+          <t>ip</t>
         </is>
       </c>
       <c r="C688" s="5" t="inlineStr">
         <is>
-          <t>DATETIME</t>
+          <t>VARCHAR(45)</t>
         </is>
       </c>
       <c r="D688" s="5" t="inlineStr">
         <is>
-          <t>예</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="E688" s="5" t="inlineStr">
@@ -23043,50 +23097,50 @@
     <row r="689">
       <c r="A689" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_port</t>
+          <t>tb_discovered_asset</t>
         </is>
       </c>
       <c r="B689" s="4" t="inlineStr">
         <is>
-          <t>discovered_port_id</t>
+          <t>hostname</t>
         </is>
       </c>
       <c r="C689" s="5" t="inlineStr">
         <is>
-          <t>BIGINT UNSIGNED</t>
+          <t>VARCHAR(255)</t>
         </is>
       </c>
       <c r="D689" s="5" t="inlineStr">
         <is>
-          <t>아니오</t>
+          <t>예</t>
         </is>
       </c>
       <c r="E689" s="5" t="inlineStr">
         <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="F689" s="5" t="inlineStr">
-        <is>
-          <t>AUTO_INCREMENT</t>
-        </is>
-      </c>
-      <c r="G689" s="3" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F689" s="5" t="inlineStr"/>
+      <c r="G689" s="3" t="inlineStr">
+        <is>
+          <t>역DNS(PTR) 호스트명. NULL=조회 실패/미조회</t>
+        </is>
+      </c>
     </row>
     <row r="690">
       <c r="A690" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_port</t>
+          <t>tb_discovered_asset</t>
         </is>
       </c>
       <c r="B690" s="4" t="inlineStr">
         <is>
-          <t>discovered_asset_id</t>
+          <t>first_seen</t>
         </is>
       </c>
       <c r="C690" s="5" t="inlineStr">
         <is>
-          <t>BIGINT UNSIGNED</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D690" s="5" t="inlineStr">
@@ -23096,7 +23150,7 @@
       </c>
       <c r="E690" s="5" t="inlineStr">
         <is>
-          <t>UNI</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F690" s="5" t="inlineStr"/>
@@ -23105,17 +23159,17 @@
     <row r="691">
       <c r="A691" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_port</t>
+          <t>tb_discovered_asset</t>
         </is>
       </c>
       <c r="B691" s="4" t="inlineStr">
         <is>
-          <t>discovery_run_id</t>
+          <t>last_seen</t>
         </is>
       </c>
       <c r="C691" s="5" t="inlineStr">
         <is>
-          <t>BIGINT UNSIGNED</t>
+          <t>DATETIME</t>
         </is>
       </c>
       <c r="D691" s="5" t="inlineStr">
@@ -23125,7 +23179,7 @@
       </c>
       <c r="E691" s="5" t="inlineStr">
         <is>
-          <t>MUL</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F691" s="5" t="inlineStr"/>
@@ -23134,22 +23188,22 @@
     <row r="692">
       <c r="A692" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_port</t>
+          <t>tb_discovered_asset</t>
         </is>
       </c>
       <c r="B692" s="4" t="inlineStr">
         <is>
-          <t>port</t>
+          <t>last_run_id</t>
         </is>
       </c>
       <c r="C692" s="5" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>BIGINT UNSIGNED</t>
         </is>
       </c>
       <c r="D692" s="5" t="inlineStr">
         <is>
-          <t>아니오</t>
+          <t>예</t>
         </is>
       </c>
       <c r="E692" s="5" t="inlineStr">
@@ -23163,55 +23217,55 @@
     <row r="693">
       <c r="A693" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_port</t>
+          <t>tb_discovered_asset</t>
         </is>
       </c>
       <c r="B693" s="4" t="inlineStr">
         <is>
-          <t>proto</t>
+          <t>host_id</t>
         </is>
       </c>
       <c r="C693" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(8)</t>
+          <t>BIGINT UNSIGNED</t>
         </is>
       </c>
       <c r="D693" s="5" t="inlineStr">
         <is>
-          <t>아니오</t>
+          <t>예</t>
         </is>
       </c>
       <c r="E693" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F693" s="5" t="inlineStr">
-        <is>
-          <t>tcp</t>
-        </is>
-      </c>
-      <c r="G693" s="3" t="inlineStr"/>
+          <t>MUL</t>
+        </is>
+      </c>
+      <c r="F693" s="5" t="inlineStr"/>
+      <c r="G693" s="3" t="inlineStr">
+        <is>
+          <t>매칭된 기존 자산(없으면 NULL=섀도우 IT 후보)</t>
+        </is>
+      </c>
     </row>
     <row r="694">
       <c r="A694" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_port</t>
+          <t>tb_discovered_asset</t>
         </is>
       </c>
       <c r="B694" s="4" t="inlineStr">
         <is>
-          <t>service_hint</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C694" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(64)</t>
+          <t>ENUM('NEW','KNOWN','IGNORED')</t>
         </is>
       </c>
       <c r="D694" s="5" t="inlineStr">
         <is>
-          <t>예</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="E694" s="5" t="inlineStr">
@@ -23219,27 +23273,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F694" s="5" t="inlineStr"/>
-      <c r="G694" s="3" t="inlineStr">
-        <is>
-          <t>포트 관례에서 유추한 서비스(추측)</t>
-        </is>
-      </c>
+      <c r="F694" s="5" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="G694" s="3" t="inlineStr"/>
     </row>
     <row r="695">
       <c r="A695" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_port</t>
+          <t>tb_discovered_asset</t>
         </is>
       </c>
       <c r="B695" s="4" t="inlineStr">
         <is>
-          <t>banner</t>
+          <t>note</t>
         </is>
       </c>
       <c r="C695" s="5" t="inlineStr">
         <is>
-          <t>VARCHAR(255)</t>
+          <t>VARCHAR(500)</t>
         </is>
       </c>
       <c r="D695" s="5" t="inlineStr">
@@ -23253,16 +23307,12 @@
         </is>
       </c>
       <c r="F695" s="5" t="inlineStr"/>
-      <c r="G695" s="3" t="inlineStr">
-        <is>
-          <t>HTTP Server 헤더 또는 TLS 인증서 CN</t>
-        </is>
-      </c>
+      <c r="G695" s="3" t="inlineStr"/>
     </row>
     <row r="696">
       <c r="A696" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_port</t>
+          <t>tb_discovered_asset</t>
         </is>
       </c>
       <c r="B696" s="4" t="inlineStr">
@@ -23295,7 +23345,7 @@
     <row r="697">
       <c r="A697" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_port</t>
+          <t>tb_discovered_asset</t>
         </is>
       </c>
       <c r="B697" s="4" t="inlineStr">
@@ -23328,7 +23378,7 @@
     <row r="698">
       <c r="A698" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_port</t>
+          <t>tb_discovered_asset</t>
         </is>
       </c>
       <c r="B698" s="4" t="inlineStr">
@@ -23361,7 +23411,7 @@
     <row r="699">
       <c r="A699" s="4" t="inlineStr">
         <is>
-          <t>tb_discovered_port</t>
+          <t>tb_discovered_asset</t>
         </is>
       </c>
       <c r="B699" s="4" t="inlineStr">
@@ -23386,6 +23436,353 @@
       </c>
       <c r="F699" s="5" t="inlineStr"/>
       <c r="G699" s="3" t="inlineStr"/>
+    </row>
+    <row r="700">
+      <c r="A700" s="4" t="inlineStr">
+        <is>
+          <t>tb_discovered_port</t>
+        </is>
+      </c>
+      <c r="B700" s="4" t="inlineStr">
+        <is>
+          <t>discovered_port_id</t>
+        </is>
+      </c>
+      <c r="C700" s="5" t="inlineStr">
+        <is>
+          <t>BIGINT UNSIGNED</t>
+        </is>
+      </c>
+      <c r="D700" s="5" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="E700" s="5" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="F700" s="5" t="inlineStr">
+        <is>
+          <t>AUTO_INCREMENT</t>
+        </is>
+      </c>
+      <c r="G700" s="3" t="inlineStr"/>
+    </row>
+    <row r="701">
+      <c r="A701" s="4" t="inlineStr">
+        <is>
+          <t>tb_discovered_port</t>
+        </is>
+      </c>
+      <c r="B701" s="4" t="inlineStr">
+        <is>
+          <t>discovered_asset_id</t>
+        </is>
+      </c>
+      <c r="C701" s="5" t="inlineStr">
+        <is>
+          <t>BIGINT UNSIGNED</t>
+        </is>
+      </c>
+      <c r="D701" s="5" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="E701" s="5" t="inlineStr">
+        <is>
+          <t>UNI</t>
+        </is>
+      </c>
+      <c r="F701" s="5" t="inlineStr"/>
+      <c r="G701" s="3" t="inlineStr"/>
+    </row>
+    <row r="702">
+      <c r="A702" s="4" t="inlineStr">
+        <is>
+          <t>tb_discovered_port</t>
+        </is>
+      </c>
+      <c r="B702" s="4" t="inlineStr">
+        <is>
+          <t>discovery_run_id</t>
+        </is>
+      </c>
+      <c r="C702" s="5" t="inlineStr">
+        <is>
+          <t>BIGINT UNSIGNED</t>
+        </is>
+      </c>
+      <c r="D702" s="5" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="E702" s="5" t="inlineStr">
+        <is>
+          <t>MUL</t>
+        </is>
+      </c>
+      <c r="F702" s="5" t="inlineStr"/>
+      <c r="G702" s="3" t="inlineStr"/>
+    </row>
+    <row r="703">
+      <c r="A703" s="4" t="inlineStr">
+        <is>
+          <t>tb_discovered_port</t>
+        </is>
+      </c>
+      <c r="B703" s="4" t="inlineStr">
+        <is>
+          <t>port</t>
+        </is>
+      </c>
+      <c r="C703" s="5" t="inlineStr">
+        <is>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="D703" s="5" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="E703" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F703" s="5" t="inlineStr"/>
+      <c r="G703" s="3" t="inlineStr"/>
+    </row>
+    <row r="704">
+      <c r="A704" s="4" t="inlineStr">
+        <is>
+          <t>tb_discovered_port</t>
+        </is>
+      </c>
+      <c r="B704" s="4" t="inlineStr">
+        <is>
+          <t>proto</t>
+        </is>
+      </c>
+      <c r="C704" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(8)</t>
+        </is>
+      </c>
+      <c r="D704" s="5" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="E704" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F704" s="5" t="inlineStr">
+        <is>
+          <t>tcp</t>
+        </is>
+      </c>
+      <c r="G704" s="3" t="inlineStr"/>
+    </row>
+    <row r="705">
+      <c r="A705" s="4" t="inlineStr">
+        <is>
+          <t>tb_discovered_port</t>
+        </is>
+      </c>
+      <c r="B705" s="4" t="inlineStr">
+        <is>
+          <t>service_hint</t>
+        </is>
+      </c>
+      <c r="C705" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(64)</t>
+        </is>
+      </c>
+      <c r="D705" s="5" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="E705" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F705" s="5" t="inlineStr"/>
+      <c r="G705" s="3" t="inlineStr">
+        <is>
+          <t>포트 관례에서 유추한 서비스(추측)</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="4" t="inlineStr">
+        <is>
+          <t>tb_discovered_port</t>
+        </is>
+      </c>
+      <c r="B706" s="4" t="inlineStr">
+        <is>
+          <t>banner</t>
+        </is>
+      </c>
+      <c r="C706" s="5" t="inlineStr">
+        <is>
+          <t>VARCHAR(255)</t>
+        </is>
+      </c>
+      <c r="D706" s="5" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="E706" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F706" s="5" t="inlineStr"/>
+      <c r="G706" s="3" t="inlineStr">
+        <is>
+          <t>HTTP Server 헤더 또는 TLS 인증서 CN</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="4" t="inlineStr">
+        <is>
+          <t>tb_discovered_port</t>
+        </is>
+      </c>
+      <c r="B707" s="4" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C707" s="5" t="inlineStr">
+        <is>
+          <t>DATETIME</t>
+        </is>
+      </c>
+      <c r="D707" s="5" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="E707" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F707" s="5" t="inlineStr">
+        <is>
+          <t>CURRENT_TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="G707" s="3" t="inlineStr"/>
+    </row>
+    <row r="708">
+      <c r="A708" s="4" t="inlineStr">
+        <is>
+          <t>tb_discovered_port</t>
+        </is>
+      </c>
+      <c r="B708" s="4" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="C708" s="5" t="inlineStr">
+        <is>
+          <t>DATETIME</t>
+        </is>
+      </c>
+      <c r="D708" s="5" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="E708" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F708" s="5" t="inlineStr">
+        <is>
+          <t>CURRENT_TIMESTAMP (ON UPDATE)</t>
+        </is>
+      </c>
+      <c r="G708" s="3" t="inlineStr"/>
+    </row>
+    <row r="709">
+      <c r="A709" s="4" t="inlineStr">
+        <is>
+          <t>tb_discovered_port</t>
+        </is>
+      </c>
+      <c r="B709" s="4" t="inlineStr">
+        <is>
+          <t>is_deleted</t>
+        </is>
+      </c>
+      <c r="C709" s="5" t="inlineStr">
+        <is>
+          <t>TINYINT(1)</t>
+        </is>
+      </c>
+      <c r="D709" s="5" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="E709" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F709" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G709" s="3" t="inlineStr"/>
+    </row>
+    <row r="710">
+      <c r="A710" s="4" t="inlineStr">
+        <is>
+          <t>tb_discovered_port</t>
+        </is>
+      </c>
+      <c r="B710" s="4" t="inlineStr">
+        <is>
+          <t>deleted_at</t>
+        </is>
+      </c>
+      <c r="C710" s="5" t="inlineStr">
+        <is>
+          <t>DATETIME</t>
+        </is>
+      </c>
+      <c r="D710" s="5" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="E710" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F710" s="5" t="inlineStr"/>
+      <c r="G710" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -23413,7 +23810,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>sha256:75518f32abc42923</t>
+          <t>sha256:4ba5c61e45adeaf7</t>
         </is>
       </c>
     </row>
@@ -23425,7 +23822,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-19T01:38:30Z</t>
+          <t>2026-08-20T14:30:44Z</t>
         </is>
       </c>
     </row>
@@ -23436,7 +23833,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>